<commit_message>
Updated default mapping of uri to @id
</commit_message>
<xml_diff>
--- a/bindings/python/tests/input/datamodels.xlsx
+++ b/bindings/python/tests/input/datamodels.xlsx
@@ -4,12 +4,13 @@
   <fileVersion lastEdited="4" lowestEdited="4" rupBuild="3820"/>
   <workbookPr date1904="0"/>
   <bookViews>
-    <workbookView activeTab="0" windowWidth="25800" windowHeight="8690"/>
+    <workbookView activeTab="0" windowWidth="25600" windowHeight="11750"/>
   </bookViews>
   <sheets>
     <sheet name="sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
+    <definedName name="id">#NAME?</definedName>
     <definedName name="_xlnm.Sheet_Title" localSheetId="0">"sheet1"</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">#REF!</definedName>
   </definedNames>
@@ -90,7 +91,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:IV4"/>
+  <dimension ref="A1:IV3"/>
   <sheetFormatPr defaultColWidth="67.5" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" style="0" width="35.1407451923077" bestFit="1" customWidth="1"/>
@@ -109,7 +110,7 @@
     <row r="1" spans="1:256">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>identifier</t>
+          <t>@id</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -483,9 +484,6 @@
         </is>
       </c>
     </row>
-    <row r="4" spans="1:256">
-      <c r="A4"/>
-    </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" selectLockedCells="1" sort="0" autoFilter="0" pivotTables="0" selectUnlockedCells="1"/>
   <printOptions/>

</xml_diff>